<commit_message>
updating trials for placing poly-U
</commit_message>
<xml_diff>
--- a/Result/LSS/Curve1_blind_sequencing_result_point_version.xlsx
+++ b/Result/LSS/Curve1_blind_sequencing_result_point_version.xlsx
@@ -1,19 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11102"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shangsilin/Desktop/Autumn 2025/mRNA_sequencing/Result/LSS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E01728B8-77CA-6148-8524-7F622BB2DADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E439DA6-3CB8-3D4F-805D-47CF734AF6E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-1600" yWindow="-21600" windowWidth="19160" windowHeight="21600" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="106 A nucleoside start" sheetId="2" r:id="rId2"/>
+    <sheet name="106 A internal start" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="75">
   <si>
     <t>base_name</t>
   </si>
@@ -226,12 +229,45 @@
   <si>
     <t>46As</t>
   </si>
+  <si>
+    <t>66As</t>
+  </si>
+  <si>
+    <t>47A</t>
+  </si>
+  <si>
+    <t>48A</t>
+  </si>
+  <si>
+    <t>49A</t>
+  </si>
+  <si>
+    <t>50A</t>
+  </si>
+  <si>
+    <t>theoretical_mass</t>
+  </si>
+  <si>
+    <t>n_position</t>
+  </si>
+  <si>
+    <t>relative_abundance</t>
+  </si>
+  <si>
+    <t>with Co</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> probably just false positives</t>
+  </si>
+  <si>
+    <t>without Co</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -247,8 +283,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Lucida Grande"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Lucida Grande"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -258,6 +307,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -274,12 +329,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -584,7 +643,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H301"/>
+  <dimension ref="A1:Q301"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -4427,7 +4486,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="193" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>9</v>
       </c>
@@ -4447,7 +4506,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="194" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>12</v>
       </c>
@@ -4467,7 +4526,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="195" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>6</v>
       </c>
@@ -4487,7 +4546,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="196" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>9</v>
       </c>
@@ -4507,7 +4566,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="197" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>11</v>
       </c>
@@ -4527,7 +4586,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="198" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>6</v>
       </c>
@@ -4547,7 +4606,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="199" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>8</v>
       </c>
@@ -4567,7 +4626,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="200" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>11</v>
       </c>
@@ -4587,7 +4646,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="201" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>8</v>
       </c>
@@ -4607,7 +4666,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="202" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>6</v>
       </c>
@@ -4627,7 +4686,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="203" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>9</v>
       </c>
@@ -4647,7 +4706,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="204" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A204" s="2" t="s">
         <v>9</v>
       </c>
@@ -4666,8 +4725,40 @@
       <c r="F204" s="2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="205" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="G204">
+        <f>B204-329.0525*20</f>
+        <v>-61.94338566514034</v>
+      </c>
+      <c r="I204">
+        <f>B204/329</f>
+        <v>19.814913721382553</v>
+      </c>
+      <c r="K204">
+        <f>(L204-18)/306</f>
+        <v>21.245098039215687</v>
+      </c>
+      <c r="L204">
+        <f>6519</f>
+        <v>6519</v>
+      </c>
+      <c r="M204">
+        <f t="shared" ref="M204:M223" si="0">(L204-18)/329</f>
+        <v>19.759878419452889</v>
+      </c>
+      <c r="O204">
+        <f>(P204-18)/306</f>
+        <v>21.245098039215687</v>
+      </c>
+      <c r="P204">
+        <f>6519</f>
+        <v>6519</v>
+      </c>
+      <c r="Q204">
+        <f>(P204-18)/329</f>
+        <v>19.759878419452889</v>
+      </c>
+    </row>
+    <row r="205" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A205" s="2" t="s">
         <v>9</v>
       </c>
@@ -4686,12 +4777,39 @@
       <c r="F205" s="2" t="s">
         <v>53</v>
       </c>
+      <c r="G205" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="H205">
-        <f t="shared" ref="H205:H250" si="0">B205-B204</f>
+        <f t="shared" ref="H205:H250" si="1">B205-B204</f>
         <v>329.0420819582605</v>
       </c>
-    </row>
-    <row r="206" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="K205">
+        <f t="shared" ref="K205:K223" si="2">(L205-18)/306</f>
+        <v>20.169934640522875</v>
+      </c>
+      <c r="L205">
+        <f>L204-329</f>
+        <v>6190</v>
+      </c>
+      <c r="M205">
+        <f t="shared" si="0"/>
+        <v>18.759878419452889</v>
+      </c>
+      <c r="O205">
+        <f t="shared" ref="O205:O225" si="3">(P205-18)/306</f>
+        <v>20.245098039215687</v>
+      </c>
+      <c r="P205">
+        <f>P204-306</f>
+        <v>6213</v>
+      </c>
+      <c r="Q205">
+        <f t="shared" ref="Q205:Q225" si="4">(P205-18)/329</f>
+        <v>18.829787234042552</v>
+      </c>
+    </row>
+    <row r="206" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A206" s="2" t="s">
         <v>9</v>
       </c>
@@ -4711,11 +4829,35 @@
         <v>53</v>
       </c>
       <c r="H206">
+        <f t="shared" si="1"/>
+        <v>329.05978735811004</v>
+      </c>
+      <c r="K206">
+        <f t="shared" si="2"/>
+        <v>19.094771241830067</v>
+      </c>
+      <c r="L206">
+        <f t="shared" ref="L206:L223" si="5">L205-329</f>
+        <v>5861</v>
+      </c>
+      <c r="M206">
         <f t="shared" si="0"/>
-        <v>329.05978735811004</v>
-      </c>
-    </row>
-    <row r="207" spans="1:8" x14ac:dyDescent="0.2">
+        <v>17.759878419452889</v>
+      </c>
+      <c r="O206">
+        <f t="shared" si="3"/>
+        <v>19.245098039215687</v>
+      </c>
+      <c r="P206">
+        <f t="shared" ref="P206:P225" si="6">P205-306</f>
+        <v>5907</v>
+      </c>
+      <c r="Q206">
+        <f t="shared" si="4"/>
+        <v>17.899696048632219</v>
+      </c>
+    </row>
+    <row r="207" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A207" s="2" t="s">
         <v>9</v>
       </c>
@@ -4735,11 +4877,35 @@
         <v>53</v>
       </c>
       <c r="H207">
+        <f t="shared" si="1"/>
+        <v>329.05162610271964</v>
+      </c>
+      <c r="K207">
+        <f t="shared" si="2"/>
+        <v>18.019607843137255</v>
+      </c>
+      <c r="L207">
+        <f t="shared" si="5"/>
+        <v>5532</v>
+      </c>
+      <c r="M207">
         <f t="shared" si="0"/>
-        <v>329.05162610271964</v>
-      </c>
-    </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.2">
+        <v>16.759878419452889</v>
+      </c>
+      <c r="O207">
+        <f t="shared" si="3"/>
+        <v>18.245098039215687</v>
+      </c>
+      <c r="P207">
+        <f t="shared" si="6"/>
+        <v>5601</v>
+      </c>
+      <c r="Q207">
+        <f t="shared" si="4"/>
+        <v>16.969604863221885</v>
+      </c>
+    </row>
+    <row r="208" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A208" s="2" t="s">
         <v>9</v>
       </c>
@@ -4759,11 +4925,35 @@
         <v>53</v>
       </c>
       <c r="H208">
+        <f t="shared" si="1"/>
+        <v>329.05156197403994</v>
+      </c>
+      <c r="K208">
+        <f t="shared" si="2"/>
+        <v>16.944444444444443</v>
+      </c>
+      <c r="L208">
+        <f t="shared" si="5"/>
+        <v>5203</v>
+      </c>
+      <c r="M208">
         <f t="shared" si="0"/>
-        <v>329.05156197403994</v>
-      </c>
-    </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.2">
+        <v>15.759878419452887</v>
+      </c>
+      <c r="O208">
+        <f t="shared" si="3"/>
+        <v>17.245098039215687</v>
+      </c>
+      <c r="P208">
+        <f t="shared" si="6"/>
+        <v>5295</v>
+      </c>
+      <c r="Q208">
+        <f t="shared" si="4"/>
+        <v>16.039513677811549</v>
+      </c>
+    </row>
+    <row r="209" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A209" s="2" t="s">
         <v>9</v>
       </c>
@@ -4783,11 +4973,35 @@
         <v>53</v>
       </c>
       <c r="H209">
+        <f t="shared" si="1"/>
+        <v>329.05770479004968</v>
+      </c>
+      <c r="K209">
+        <f t="shared" si="2"/>
+        <v>15.869281045751634</v>
+      </c>
+      <c r="L209">
+        <f t="shared" si="5"/>
+        <v>4874</v>
+      </c>
+      <c r="M209">
         <f t="shared" si="0"/>
-        <v>329.05770479004968</v>
-      </c>
-    </row>
-    <row r="210" spans="1:8" x14ac:dyDescent="0.2">
+        <v>14.759878419452887</v>
+      </c>
+      <c r="O209">
+        <f t="shared" si="3"/>
+        <v>16.245098039215687</v>
+      </c>
+      <c r="P209">
+        <f t="shared" si="6"/>
+        <v>4989</v>
+      </c>
+      <c r="Q209">
+        <f t="shared" si="4"/>
+        <v>15.109422492401215</v>
+      </c>
+    </row>
+    <row r="210" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A210" s="2" t="s">
         <v>9</v>
       </c>
@@ -4807,11 +5021,35 @@
         <v>53</v>
       </c>
       <c r="H210">
+        <f t="shared" si="1"/>
+        <v>329.0424975549704</v>
+      </c>
+      <c r="K210">
+        <f t="shared" si="2"/>
+        <v>14.794117647058824</v>
+      </c>
+      <c r="L210">
+        <f t="shared" si="5"/>
+        <v>4545</v>
+      </c>
+      <c r="M210">
         <f t="shared" si="0"/>
-        <v>329.0424975549704</v>
-      </c>
-    </row>
-    <row r="211" spans="1:8" x14ac:dyDescent="0.2">
+        <v>13.759878419452887</v>
+      </c>
+      <c r="O210">
+        <f t="shared" si="3"/>
+        <v>15.245098039215685</v>
+      </c>
+      <c r="P210">
+        <f t="shared" si="6"/>
+        <v>4683</v>
+      </c>
+      <c r="Q210">
+        <f t="shared" si="4"/>
+        <v>14.179331306990882</v>
+      </c>
+    </row>
+    <row r="211" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A211" s="2" t="s">
         <v>9</v>
       </c>
@@ -4831,11 +5069,35 @@
         <v>53</v>
       </c>
       <c r="H211">
+        <f t="shared" si="1"/>
+        <v>329.0572325610392</v>
+      </c>
+      <c r="K211">
+        <f t="shared" si="2"/>
+        <v>13.718954248366012</v>
+      </c>
+      <c r="L211">
+        <f t="shared" si="5"/>
+        <v>4216</v>
+      </c>
+      <c r="M211">
         <f t="shared" si="0"/>
-        <v>329.0572325610392</v>
-      </c>
-    </row>
-    <row r="212" spans="1:8" x14ac:dyDescent="0.2">
+        <v>12.759878419452887</v>
+      </c>
+      <c r="O211">
+        <f t="shared" si="3"/>
+        <v>14.245098039215685</v>
+      </c>
+      <c r="P211">
+        <f t="shared" si="6"/>
+        <v>4377</v>
+      </c>
+      <c r="Q211">
+        <f t="shared" si="4"/>
+        <v>13.249240121580547</v>
+      </c>
+    </row>
+    <row r="212" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A212" s="2" t="s">
         <v>9</v>
       </c>
@@ -4855,11 +5117,35 @@
         <v>53</v>
       </c>
       <c r="H212">
+        <f t="shared" si="1"/>
+        <v>329.04302245746112</v>
+      </c>
+      <c r="K212">
+        <f t="shared" si="2"/>
+        <v>12.643790849673202</v>
+      </c>
+      <c r="L212">
+        <f t="shared" si="5"/>
+        <v>3887</v>
+      </c>
+      <c r="M212">
         <f t="shared" si="0"/>
-        <v>329.04302245746112</v>
-      </c>
-    </row>
-    <row r="213" spans="1:8" x14ac:dyDescent="0.2">
+        <v>11.759878419452887</v>
+      </c>
+      <c r="O212">
+        <f t="shared" si="3"/>
+        <v>13.245098039215685</v>
+      </c>
+      <c r="P212">
+        <f t="shared" si="6"/>
+        <v>4071</v>
+      </c>
+      <c r="Q212">
+        <f t="shared" si="4"/>
+        <v>12.319148936170214</v>
+      </c>
+    </row>
+    <row r="213" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A213" s="2" t="s">
         <v>9</v>
       </c>
@@ -4879,11 +5165,35 @@
         <v>53</v>
       </c>
       <c r="H213">
+        <f t="shared" si="1"/>
+        <v>329.06196379410903</v>
+      </c>
+      <c r="K213">
+        <f t="shared" si="2"/>
+        <v>11.568627450980392</v>
+      </c>
+      <c r="L213">
+        <f t="shared" si="5"/>
+        <v>3558</v>
+      </c>
+      <c r="M213">
         <f t="shared" si="0"/>
-        <v>329.06196379410903</v>
-      </c>
-    </row>
-    <row r="214" spans="1:8" x14ac:dyDescent="0.2">
+        <v>10.759878419452887</v>
+      </c>
+      <c r="O213">
+        <f t="shared" si="3"/>
+        <v>12.245098039215685</v>
+      </c>
+      <c r="P213">
+        <f t="shared" si="6"/>
+        <v>3765</v>
+      </c>
+      <c r="Q213">
+        <f t="shared" si="4"/>
+        <v>11.389057750759878</v>
+      </c>
+    </row>
+    <row r="214" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A214" s="2" t="s">
         <v>9</v>
       </c>
@@ -4903,11 +5213,35 @@
         <v>53</v>
       </c>
       <c r="H214">
+        <f t="shared" si="1"/>
+        <v>329.04758816923095</v>
+      </c>
+      <c r="K214">
+        <f t="shared" si="2"/>
+        <v>10.493464052287582</v>
+      </c>
+      <c r="L214">
+        <f t="shared" si="5"/>
+        <v>3229</v>
+      </c>
+      <c r="M214">
         <f t="shared" si="0"/>
-        <v>329.04758816923095</v>
-      </c>
-    </row>
-    <row r="215" spans="1:8" x14ac:dyDescent="0.2">
+        <v>9.7598784194528871</v>
+      </c>
+      <c r="O214">
+        <f t="shared" si="3"/>
+        <v>11.245098039215685</v>
+      </c>
+      <c r="P214">
+        <f t="shared" si="6"/>
+        <v>3459</v>
+      </c>
+      <c r="Q214">
+        <f t="shared" si="4"/>
+        <v>10.458966565349543</v>
+      </c>
+    </row>
+    <row r="215" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A215" s="2" t="s">
         <v>9</v>
       </c>
@@ -4927,11 +5261,35 @@
         <v>53</v>
       </c>
       <c r="H215">
+        <f t="shared" si="1"/>
+        <v>329.06478558024901</v>
+      </c>
+      <c r="K215">
+        <f t="shared" si="2"/>
+        <v>9.4183006535947715</v>
+      </c>
+      <c r="L215">
+        <f t="shared" si="5"/>
+        <v>2900</v>
+      </c>
+      <c r="M215">
         <f t="shared" si="0"/>
-        <v>329.06478558024901</v>
-      </c>
-    </row>
-    <row r="216" spans="1:8" x14ac:dyDescent="0.2">
+        <v>8.7598784194528871</v>
+      </c>
+      <c r="O215">
+        <f t="shared" si="3"/>
+        <v>10.245098039215685</v>
+      </c>
+      <c r="P215">
+        <f t="shared" si="6"/>
+        <v>3153</v>
+      </c>
+      <c r="Q215">
+        <f t="shared" si="4"/>
+        <v>9.5288753799392101</v>
+      </c>
+    </row>
+    <row r="216" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A216" s="2" t="s">
         <v>9</v>
       </c>
@@ -4951,11 +5309,35 @@
         <v>53</v>
       </c>
       <c r="H216">
+        <f t="shared" si="1"/>
+        <v>329.04869343410064</v>
+      </c>
+      <c r="K216">
+        <f t="shared" si="2"/>
+        <v>8.3431372549019613</v>
+      </c>
+      <c r="L216">
+        <f t="shared" si="5"/>
+        <v>2571</v>
+      </c>
+      <c r="M216">
         <f t="shared" si="0"/>
-        <v>329.04869343410064</v>
-      </c>
-    </row>
-    <row r="217" spans="1:8" x14ac:dyDescent="0.2">
+        <v>7.7598784194528871</v>
+      </c>
+      <c r="O216">
+        <f t="shared" si="3"/>
+        <v>9.2450980392156854</v>
+      </c>
+      <c r="P216">
+        <f t="shared" si="6"/>
+        <v>2847</v>
+      </c>
+      <c r="Q216">
+        <f t="shared" si="4"/>
+        <v>8.598784194528875</v>
+      </c>
+    </row>
+    <row r="217" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A217" s="2" t="s">
         <v>9</v>
       </c>
@@ -4975,11 +5357,35 @@
         <v>53</v>
       </c>
       <c r="H217">
+        <f t="shared" si="1"/>
+        <v>329.05141851420012</v>
+      </c>
+      <c r="K217">
+        <f t="shared" si="2"/>
+        <v>7.2679738562091503</v>
+      </c>
+      <c r="L217">
+        <f t="shared" si="5"/>
+        <v>2242</v>
+      </c>
+      <c r="M217">
         <f t="shared" si="0"/>
-        <v>329.05141851420012</v>
-      </c>
-    </row>
-    <row r="218" spans="1:8" x14ac:dyDescent="0.2">
+        <v>6.7598784194528871</v>
+      </c>
+      <c r="O217">
+        <f t="shared" si="3"/>
+        <v>8.2450980392156854</v>
+      </c>
+      <c r="P217">
+        <f t="shared" si="6"/>
+        <v>2541</v>
+      </c>
+      <c r="Q217">
+        <f t="shared" si="4"/>
+        <v>7.6686930091185408</v>
+      </c>
+    </row>
+    <row r="218" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A218" s="2" t="s">
         <v>9</v>
       </c>
@@ -4999,11 +5405,35 @@
         <v>53</v>
       </c>
       <c r="H218">
+        <f t="shared" si="1"/>
+        <v>329.07069458200021</v>
+      </c>
+      <c r="K218">
+        <f t="shared" si="2"/>
+        <v>6.1928104575163401</v>
+      </c>
+      <c r="L218">
+        <f t="shared" si="5"/>
+        <v>1913</v>
+      </c>
+      <c r="M218">
         <f t="shared" si="0"/>
-        <v>329.07069458200021</v>
-      </c>
-    </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.2">
+        <v>5.7598784194528871</v>
+      </c>
+      <c r="O218">
+        <f t="shared" si="3"/>
+        <v>7.2450980392156863</v>
+      </c>
+      <c r="P218">
+        <f t="shared" si="6"/>
+        <v>2235</v>
+      </c>
+      <c r="Q218">
+        <f t="shared" si="4"/>
+        <v>6.7386018237082066</v>
+      </c>
+    </row>
+    <row r="219" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A219" s="2" t="s">
         <v>8</v>
       </c>
@@ -5023,11 +5453,35 @@
         <v>53</v>
       </c>
       <c r="H219">
+        <f t="shared" si="1"/>
+        <v>329.03548825920006</v>
+      </c>
+      <c r="K219">
+        <f t="shared" si="2"/>
+        <v>5.117647058823529</v>
+      </c>
+      <c r="L219">
+        <f t="shared" si="5"/>
+        <v>1584</v>
+      </c>
+      <c r="M219">
         <f t="shared" si="0"/>
-        <v>329.03548825920006</v>
-      </c>
-    </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.2">
+        <v>4.7598784194528871</v>
+      </c>
+      <c r="O219">
+        <f t="shared" si="3"/>
+        <v>6.2450980392156863</v>
+      </c>
+      <c r="P219">
+        <f t="shared" si="6"/>
+        <v>1929</v>
+      </c>
+      <c r="Q219">
+        <f t="shared" si="4"/>
+        <v>5.8085106382978724</v>
+      </c>
+    </row>
+    <row r="220" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A220" s="2" t="s">
         <v>9</v>
       </c>
@@ -5047,11 +5501,35 @@
         <v>53</v>
       </c>
       <c r="H220">
+        <f t="shared" si="1"/>
+        <v>329.05268754749886</v>
+      </c>
+      <c r="K220">
+        <f t="shared" si="2"/>
+        <v>4.0424836601307188</v>
+      </c>
+      <c r="L220">
+        <f t="shared" si="5"/>
+        <v>1255</v>
+      </c>
+      <c r="M220">
         <f t="shared" si="0"/>
-        <v>329.05268754749886</v>
-      </c>
-    </row>
-    <row r="221" spans="1:8" x14ac:dyDescent="0.2">
+        <v>3.7598784194528876</v>
+      </c>
+      <c r="O220">
+        <f t="shared" si="3"/>
+        <v>5.2450980392156863</v>
+      </c>
+      <c r="P220">
+        <f t="shared" si="6"/>
+        <v>1623</v>
+      </c>
+      <c r="Q220">
+        <f t="shared" si="4"/>
+        <v>4.8784194528875382</v>
+      </c>
+    </row>
+    <row r="221" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A221" s="2" t="s">
         <v>9</v>
       </c>
@@ -5071,11 +5549,35 @@
         <v>53</v>
       </c>
       <c r="H221">
+        <f t="shared" si="1"/>
+        <v>329.05662086850134</v>
+      </c>
+      <c r="K221">
+        <f t="shared" si="2"/>
+        <v>2.9673202614379086</v>
+      </c>
+      <c r="L221">
+        <f t="shared" si="5"/>
+        <v>926</v>
+      </c>
+      <c r="M221">
         <f t="shared" si="0"/>
-        <v>329.05662086850134</v>
-      </c>
-    </row>
-    <row r="222" spans="1:8" x14ac:dyDescent="0.2">
+        <v>2.7598784194528876</v>
+      </c>
+      <c r="O221">
+        <f t="shared" si="3"/>
+        <v>4.2450980392156863</v>
+      </c>
+      <c r="P221">
+        <f t="shared" si="6"/>
+        <v>1317</v>
+      </c>
+      <c r="Q221">
+        <f t="shared" si="4"/>
+        <v>3.9483282674772036</v>
+      </c>
+    </row>
+    <row r="222" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A222" s="2" t="s">
         <v>9</v>
       </c>
@@ -5095,11 +5597,35 @@
         <v>53</v>
       </c>
       <c r="H222">
+        <f t="shared" si="1"/>
+        <v>329.06198928159938</v>
+      </c>
+      <c r="K222">
+        <f t="shared" si="2"/>
+        <v>1.892156862745098</v>
+      </c>
+      <c r="L222">
+        <f t="shared" si="5"/>
+        <v>597</v>
+      </c>
+      <c r="M222">
         <f t="shared" si="0"/>
-        <v>329.06198928159938</v>
-      </c>
-    </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.2">
+        <v>1.7598784194528876</v>
+      </c>
+      <c r="O222">
+        <f t="shared" si="3"/>
+        <v>3.2450980392156863</v>
+      </c>
+      <c r="P222">
+        <f t="shared" si="6"/>
+        <v>1011</v>
+      </c>
+      <c r="Q222">
+        <f t="shared" si="4"/>
+        <v>3.0182370820668694</v>
+      </c>
+    </row>
+    <row r="223" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A223" s="2" t="s">
         <v>9</v>
       </c>
@@ -5119,11 +5645,35 @@
         <v>53</v>
       </c>
       <c r="H223">
+        <f t="shared" si="1"/>
+        <v>329.02704211140008</v>
+      </c>
+      <c r="K223">
+        <f t="shared" si="2"/>
+        <v>0.81699346405228757</v>
+      </c>
+      <c r="L223">
+        <f t="shared" si="5"/>
+        <v>268</v>
+      </c>
+      <c r="M223">
         <f t="shared" si="0"/>
-        <v>329.02704211140008</v>
-      </c>
-    </row>
-    <row r="224" spans="1:8" x14ac:dyDescent="0.2">
+        <v>0.75987841945288759</v>
+      </c>
+      <c r="O223">
+        <f t="shared" si="3"/>
+        <v>2.2450980392156863</v>
+      </c>
+      <c r="P223">
+        <f t="shared" si="6"/>
+        <v>705</v>
+      </c>
+      <c r="Q223">
+        <f t="shared" si="4"/>
+        <v>2.0881458966565352</v>
+      </c>
+    </row>
+    <row r="224" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A224" s="2" t="s">
         <v>9</v>
       </c>
@@ -5143,11 +5693,23 @@
         <v>53</v>
       </c>
       <c r="H224">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.06068805389987</v>
       </c>
-    </row>
-    <row r="225" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="O224">
+        <f t="shared" si="3"/>
+        <v>1.2450980392156863</v>
+      </c>
+      <c r="P224">
+        <f t="shared" si="6"/>
+        <v>399</v>
+      </c>
+      <c r="Q224">
+        <f t="shared" si="4"/>
+        <v>1.1580547112462005</v>
+      </c>
+    </row>
+    <row r="225" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A225" s="2" t="s">
         <v>9</v>
       </c>
@@ -5167,11 +5729,23 @@
         <v>53</v>
       </c>
       <c r="H225">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.06905560899941</v>
       </c>
-    </row>
-    <row r="226" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="O225">
+        <f t="shared" si="3"/>
+        <v>0.24509803921568626</v>
+      </c>
+      <c r="P225">
+        <f t="shared" si="6"/>
+        <v>93</v>
+      </c>
+      <c r="Q225">
+        <f t="shared" si="4"/>
+        <v>0.22796352583586627</v>
+      </c>
+    </row>
+    <row r="226" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A226" s="2" t="s">
         <v>9</v>
       </c>
@@ -5191,11 +5765,11 @@
         <v>53</v>
       </c>
       <c r="H226">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.03133953680117</v>
       </c>
     </row>
-    <row r="227" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A227" s="2" t="s">
         <v>9</v>
       </c>
@@ -5215,11 +5789,11 @@
         <v>53</v>
       </c>
       <c r="H227">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.05734280029901</v>
       </c>
     </row>
-    <row r="228" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A228" s="2" t="s">
         <v>9</v>
       </c>
@@ -5239,11 +5813,11 @@
         <v>53</v>
       </c>
       <c r="H228">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.06201590159981</v>
       </c>
     </row>
-    <row r="229" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A229" s="2" t="s">
         <v>9</v>
       </c>
@@ -5263,11 +5837,11 @@
         <v>53</v>
       </c>
       <c r="H229">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.0664990542009</v>
       </c>
     </row>
-    <row r="230" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A230" s="2" t="s">
         <v>9</v>
       </c>
@@ -5287,11 +5861,11 @@
         <v>53</v>
       </c>
       <c r="H230">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.04115929040017</v>
       </c>
     </row>
-    <row r="231" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A231" s="2" t="s">
         <v>9</v>
       </c>
@@ -5311,11 +5885,11 @@
         <v>53</v>
       </c>
       <c r="H231">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.0566548275001</v>
       </c>
     </row>
-    <row r="232" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A232" s="2" t="s">
         <v>9</v>
       </c>
@@ -5335,11 +5909,11 @@
         <v>53</v>
       </c>
       <c r="H232">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.05071181099993</v>
       </c>
     </row>
-    <row r="233" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A233" s="2" t="s">
         <v>9</v>
       </c>
@@ -5359,11 +5933,11 @@
         <v>53</v>
       </c>
       <c r="H233">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.05407485189971</v>
       </c>
     </row>
-    <row r="234" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A234" s="2" t="s">
         <v>9</v>
       </c>
@@ -5383,11 +5957,11 @@
         <v>53</v>
       </c>
       <c r="H234">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.05171547030113</v>
       </c>
     </row>
-    <row r="235" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A235" s="2" t="s">
         <v>9</v>
       </c>
@@ -5407,11 +5981,11 @@
         <v>53</v>
       </c>
       <c r="H235">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.03965414709819</v>
       </c>
     </row>
-    <row r="236" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A236" s="2" t="s">
         <v>9</v>
       </c>
@@ -5431,11 +6005,11 @@
         <v>53</v>
       </c>
       <c r="H236">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.06265461369912</v>
       </c>
     </row>
-    <row r="237" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A237" s="2" t="s">
         <v>9</v>
       </c>
@@ -5455,11 +6029,11 @@
         <v>53</v>
       </c>
       <c r="H237">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.05822904399975</v>
       </c>
     </row>
-    <row r="238" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A238" s="2" t="s">
         <v>9</v>
       </c>
@@ -5479,11 +6053,11 @@
         <v>53</v>
       </c>
       <c r="H238">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.05044541080133</v>
       </c>
     </row>
-    <row r="239" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A239" s="2" t="s">
         <v>9</v>
       </c>
@@ -5503,11 +6077,11 @@
         <v>53</v>
       </c>
       <c r="H239">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.03998828190015</v>
       </c>
     </row>
-    <row r="240" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A240" s="2" t="s">
         <v>9</v>
       </c>
@@ -5527,11 +6101,11 @@
         <v>53</v>
       </c>
       <c r="H240">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.06093416990188</v>
       </c>
     </row>
-    <row r="241" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A241" s="2" t="s">
         <v>9</v>
       </c>
@@ -5551,11 +6125,11 @@
         <v>53</v>
       </c>
       <c r="H241">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.05425163379914</v>
       </c>
     </row>
-    <row r="242" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A242" s="2" t="s">
         <v>9</v>
       </c>
@@ -5575,11 +6149,11 @@
         <v>53</v>
       </c>
       <c r="H242">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.05700442869784</v>
       </c>
     </row>
-    <row r="243" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A243" s="2" t="s">
         <v>9</v>
       </c>
@@ -5599,11 +6173,11 @@
         <v>53</v>
       </c>
       <c r="H243">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.05375325600107</v>
       </c>
     </row>
-    <row r="244" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A244" s="2" t="s">
         <v>9</v>
       </c>
@@ -5623,11 +6197,11 @@
         <v>53</v>
       </c>
       <c r="H244">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.0489404182008</v>
       </c>
     </row>
-    <row r="245" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A245" s="2" t="s">
         <v>9</v>
       </c>
@@ -5647,11 +6221,11 @@
         <v>53</v>
       </c>
       <c r="H245">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.05247268590028</v>
       </c>
     </row>
-    <row r="246" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A246" s="2" t="s">
         <v>9</v>
       </c>
@@ -5671,11 +6245,11 @@
         <v>53</v>
       </c>
       <c r="H246">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.03989707840083</v>
       </c>
     </row>
-    <row r="247" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A247" s="2" t="s">
         <v>9</v>
       </c>
@@ -5695,11 +6269,11 @@
         <v>53</v>
       </c>
       <c r="H247">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.06975582499945</v>
       </c>
     </row>
-    <row r="248" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A248" s="2" t="s">
         <v>9</v>
       </c>
@@ -5719,11 +6293,11 @@
         <v>53</v>
       </c>
       <c r="H248">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.03648248709942</v>
       </c>
     </row>
-    <row r="249" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A249" s="2" t="s">
         <v>9</v>
       </c>
@@ -5743,11 +6317,11 @@
         <v>53</v>
       </c>
       <c r="H249">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.0611278619981</v>
       </c>
     </row>
-    <row r="250" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A250" s="2" t="s">
         <v>9</v>
       </c>
@@ -5770,11 +6344,18 @@
         <v>63</v>
       </c>
       <c r="H250">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>329.04745745960099</v>
       </c>
-    </row>
-    <row r="251" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I250">
+        <f>B250+329.0525</f>
+        <v>21984.577907242601</v>
+      </c>
+      <c r="J250" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="251" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>8</v>
       </c>
@@ -5793,8 +6374,15 @@
       <c r="F251" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="252" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I251">
+        <f>I250+329.0525</f>
+        <v>22313.630407242603</v>
+      </c>
+      <c r="J251" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="252" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
         <v>11</v>
       </c>
@@ -5813,8 +6401,15 @@
       <c r="F252" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="253" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I252">
+        <f>I251+329.0525</f>
+        <v>22642.682907242604</v>
+      </c>
+      <c r="J252" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="253" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
         <v>6</v>
       </c>
@@ -5833,8 +6428,15 @@
       <c r="F253" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="254" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I253">
+        <f>I252+329.0525</f>
+        <v>22971.735407242606</v>
+      </c>
+      <c r="J253" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="254" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
         <v>9</v>
       </c>
@@ -5853,8 +6455,12 @@
       <c r="F254" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="255" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I254">
+        <f t="shared" ref="I254:I258" si="7">I253+329.0525</f>
+        <v>23300.787907242608</v>
+      </c>
+    </row>
+    <row r="255" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
         <v>6</v>
       </c>
@@ -5873,8 +6479,12 @@
       <c r="F255" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="256" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I255">
+        <f t="shared" si="7"/>
+        <v>23629.840407242609</v>
+      </c>
+    </row>
+    <row r="256" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
         <v>6</v>
       </c>
@@ -5893,8 +6503,12 @@
       <c r="F256" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="257" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I256">
+        <f t="shared" si="7"/>
+        <v>23958.892907242611</v>
+      </c>
+    </row>
+    <row r="257" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
         <v>8</v>
       </c>
@@ -5913,8 +6527,12 @@
       <c r="F257" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="258" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I257">
+        <f t="shared" si="7"/>
+        <v>24287.945407242612</v>
+      </c>
+    </row>
+    <row r="258" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
         <v>11</v>
       </c>
@@ -5933,8 +6551,12 @@
       <c r="F258" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="259" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I258">
+        <f t="shared" si="7"/>
+        <v>24616.997907242614</v>
+      </c>
+    </row>
+    <row r="259" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
         <v>11</v>
       </c>
@@ -5954,7 +6576,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="260" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A260" t="s">
         <v>11</v>
       </c>
@@ -5974,7 +6596,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="261" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A261" t="s">
         <v>6</v>
       </c>
@@ -5994,7 +6616,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="262" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A262" t="s">
         <v>9</v>
       </c>
@@ -6014,7 +6636,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="263" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A263" t="s">
         <v>8</v>
       </c>
@@ -6034,7 +6656,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A264" t="s">
         <v>9</v>
       </c>
@@ -6054,7 +6676,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="265" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A265" t="s">
         <v>11</v>
       </c>
@@ -6074,7 +6696,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="266" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A266" t="s">
         <v>9</v>
       </c>
@@ -6094,7 +6716,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="267" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A267" t="s">
         <v>6</v>
       </c>
@@ -6114,7 +6736,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="268" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A268" t="s">
         <v>9</v>
       </c>
@@ -6134,7 +6756,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="269" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A269" t="s">
         <v>8</v>
       </c>
@@ -6154,7 +6776,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="270" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A270" t="s">
         <v>9</v>
       </c>
@@ -6174,7 +6796,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="271" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A271" t="s">
         <v>12</v>
       </c>
@@ -6194,7 +6816,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="272" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A272" t="s">
         <v>9</v>
       </c>
@@ -6792,6 +7414,2305 @@
       </c>
       <c r="F301" t="s">
         <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC340402-EED3-384C-9B97-36B30EF6DD66}">
+  <dimension ref="A1:G57"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="5">
+        <v>2570.4639999999999</v>
+      </c>
+      <c r="C2" s="5">
+        <v>8</v>
+      </c>
+      <c r="D2" s="5">
+        <v>2570.4690000000001</v>
+      </c>
+      <c r="E2" s="5">
+        <v>6195.54</v>
+      </c>
+      <c r="F2" s="5">
+        <v>4.0509120000000003</v>
+      </c>
+      <c r="G2" s="5">
+        <v>0.17677109999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="5">
+        <v>3886.674</v>
+      </c>
+      <c r="C3" s="5">
+        <v>12</v>
+      </c>
+      <c r="D3" s="5">
+        <v>3886.6849999999999</v>
+      </c>
+      <c r="E3" s="5">
+        <v>43666.54</v>
+      </c>
+      <c r="F3" s="5">
+        <v>8.0111070000000009</v>
+      </c>
+      <c r="G3" s="5">
+        <v>1.2458937000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="5">
+        <v>4215.7269999999999</v>
+      </c>
+      <c r="C4" s="5">
+        <v>13</v>
+      </c>
+      <c r="D4" s="5">
+        <v>4215.7389999999996</v>
+      </c>
+      <c r="E4" s="5">
+        <v>66024.47</v>
+      </c>
+      <c r="F4" s="5">
+        <v>8.6721979999999999</v>
+      </c>
+      <c r="G4" s="5">
+        <v>1.8838101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="5">
+        <v>4544.7790000000005</v>
+      </c>
+      <c r="C5" s="5">
+        <v>14</v>
+      </c>
+      <c r="D5" s="5">
+        <v>4544.79</v>
+      </c>
+      <c r="E5" s="5">
+        <v>106821.14</v>
+      </c>
+      <c r="F5" s="5">
+        <v>9.2432259999999999</v>
+      </c>
+      <c r="G5" s="5">
+        <v>3.0478206000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="5">
+        <v>4873.8320000000003</v>
+      </c>
+      <c r="C6" s="5">
+        <v>15</v>
+      </c>
+      <c r="D6" s="5">
+        <v>4873.84</v>
+      </c>
+      <c r="E6" s="5">
+        <v>118046.38</v>
+      </c>
+      <c r="F6" s="5">
+        <v>9.7780419999999992</v>
+      </c>
+      <c r="G6" s="5">
+        <v>3.3680992000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="5">
+        <v>5202.884</v>
+      </c>
+      <c r="C7" s="5">
+        <v>16</v>
+      </c>
+      <c r="D7" s="5">
+        <v>5202.8890000000001</v>
+      </c>
+      <c r="E7" s="5">
+        <v>137243.29999999999</v>
+      </c>
+      <c r="F7" s="5">
+        <v>10.258682</v>
+      </c>
+      <c r="G7" s="5">
+        <v>3.9158257000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="5">
+        <v>5531.9369999999999</v>
+      </c>
+      <c r="C8" s="5">
+        <v>17</v>
+      </c>
+      <c r="D8" s="5">
+        <v>5531.9350000000004</v>
+      </c>
+      <c r="E8" s="5">
+        <v>76618.91</v>
+      </c>
+      <c r="F8" s="5">
+        <v>10.712296</v>
+      </c>
+      <c r="G8" s="5">
+        <v>2.1860906</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="5">
+        <v>5860.9889999999996</v>
+      </c>
+      <c r="C9" s="5">
+        <v>18</v>
+      </c>
+      <c r="D9" s="5">
+        <v>5860.9960000000001</v>
+      </c>
+      <c r="E9" s="5">
+        <v>81104.33</v>
+      </c>
+      <c r="F9" s="5">
+        <v>11.102497</v>
+      </c>
+      <c r="G9" s="5">
+        <v>2.3140686000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5">
+        <v>6519.0940000000001</v>
+      </c>
+      <c r="C10" s="5">
+        <v>20</v>
+      </c>
+      <c r="D10" s="5">
+        <v>6519.107</v>
+      </c>
+      <c r="E10" s="5">
+        <v>34352.19</v>
+      </c>
+      <c r="F10" s="5">
+        <v>11.792285</v>
+      </c>
+      <c r="G10" s="5">
+        <v>0.98013660000000002</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="5">
+        <v>6848.1469999999999</v>
+      </c>
+      <c r="C11" s="5">
+        <v>21</v>
+      </c>
+      <c r="D11" s="5">
+        <v>6848.1490000000003</v>
+      </c>
+      <c r="E11" s="5">
+        <v>30790.84</v>
+      </c>
+      <c r="F11" s="5">
+        <v>12.091965</v>
+      </c>
+      <c r="G11" s="5">
+        <v>0.87852419999999998</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="5">
+        <v>7177.1989999999996</v>
+      </c>
+      <c r="C12" s="5">
+        <v>22</v>
+      </c>
+      <c r="D12" s="5">
+        <v>7177.2079999999996</v>
+      </c>
+      <c r="E12" s="5">
+        <v>25726.880000000001</v>
+      </c>
+      <c r="F12" s="5">
+        <v>12.391660999999999</v>
+      </c>
+      <c r="G12" s="5">
+        <v>0.73403929999999995</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="5">
+        <v>7506.2520000000004</v>
+      </c>
+      <c r="C13" s="5">
+        <v>23</v>
+      </c>
+      <c r="D13" s="5">
+        <v>7506.26</v>
+      </c>
+      <c r="E13" s="5">
+        <v>32436.71</v>
+      </c>
+      <c r="F13" s="5">
+        <v>12.659433</v>
+      </c>
+      <c r="G13" s="5">
+        <v>0.92548419999999998</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="5">
+        <v>7835.3040000000001</v>
+      </c>
+      <c r="C14" s="5">
+        <v>24</v>
+      </c>
+      <c r="D14" s="5">
+        <v>7835.3119999999999</v>
+      </c>
+      <c r="E14" s="5">
+        <v>34052.120000000003</v>
+      </c>
+      <c r="F14" s="5">
+        <v>12.900062999999999</v>
+      </c>
+      <c r="G14" s="5">
+        <v>0.97157499999999997</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" s="5">
+        <v>8164.357</v>
+      </c>
+      <c r="C15" s="5">
+        <v>25</v>
+      </c>
+      <c r="D15" s="5">
+        <v>8164.3689999999997</v>
+      </c>
+      <c r="E15" s="5">
+        <v>27038.59</v>
+      </c>
+      <c r="F15" s="5">
+        <v>13.140724000000001</v>
+      </c>
+      <c r="G15" s="5">
+        <v>0.77146499999999996</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="5">
+        <v>8493.4089999999997</v>
+      </c>
+      <c r="C16" s="5">
+        <v>26</v>
+      </c>
+      <c r="D16" s="5">
+        <v>8493.4120000000003</v>
+      </c>
+      <c r="E16" s="5">
+        <v>32253.53</v>
+      </c>
+      <c r="F16" s="5">
+        <v>13.381479000000001</v>
+      </c>
+      <c r="G16" s="5">
+        <v>0.92025769999999996</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="5">
+        <v>8822.4619999999995</v>
+      </c>
+      <c r="C17" s="5">
+        <v>27</v>
+      </c>
+      <c r="D17" s="5">
+        <v>8822.4689999999991</v>
+      </c>
+      <c r="E17" s="5">
+        <v>18314.3</v>
+      </c>
+      <c r="F17" s="5">
+        <v>13.563162</v>
+      </c>
+      <c r="G17" s="5">
+        <v>0.5225436</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="5">
+        <v>9151.5139999999992</v>
+      </c>
+      <c r="C18" s="5">
+        <v>28</v>
+      </c>
+      <c r="D18" s="5">
+        <v>9151.5120000000006</v>
+      </c>
+      <c r="E18" s="5">
+        <v>25846.54</v>
+      </c>
+      <c r="F18" s="5">
+        <v>13.740375</v>
+      </c>
+      <c r="G18" s="5">
+        <v>0.73745340000000004</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" s="5">
+        <v>9480.5669999999991</v>
+      </c>
+      <c r="C19" s="5">
+        <v>29</v>
+      </c>
+      <c r="D19" s="5">
+        <v>9480.5740000000005</v>
+      </c>
+      <c r="E19" s="5">
+        <v>32379.66</v>
+      </c>
+      <c r="F19" s="5">
+        <v>13.917571000000001</v>
+      </c>
+      <c r="G19" s="5">
+        <v>0.92385640000000002</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="5">
+        <v>9809.6190000000006</v>
+      </c>
+      <c r="C20" s="5">
+        <v>30</v>
+      </c>
+      <c r="D20" s="5">
+        <v>9809.6219999999994</v>
+      </c>
+      <c r="E20" s="5">
+        <v>37334.720000000001</v>
+      </c>
+      <c r="F20" s="5">
+        <v>14.099273</v>
+      </c>
+      <c r="G20" s="5">
+        <v>1.0652341999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21" s="5">
+        <v>10138.672</v>
+      </c>
+      <c r="C21" s="5">
+        <v>31</v>
+      </c>
+      <c r="D21" s="5">
+        <v>10138.686</v>
+      </c>
+      <c r="E21" s="5">
+        <v>39796.11</v>
+      </c>
+      <c r="F21" s="5">
+        <v>14.2492</v>
+      </c>
+      <c r="G21" s="5">
+        <v>1.1354626000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" s="5">
+        <v>10467.724</v>
+      </c>
+      <c r="C22" s="5">
+        <v>32</v>
+      </c>
+      <c r="D22" s="5">
+        <v>10467.735000000001</v>
+      </c>
+      <c r="E22" s="5">
+        <v>45816.76</v>
+      </c>
+      <c r="F22" s="5">
+        <v>14.399145000000001</v>
+      </c>
+      <c r="G22" s="5">
+        <v>1.3072436999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="5">
+        <v>10796.777</v>
+      </c>
+      <c r="C23" s="5">
+        <v>33</v>
+      </c>
+      <c r="D23" s="5">
+        <v>10796.787</v>
+      </c>
+      <c r="E23" s="5">
+        <v>43869.38</v>
+      </c>
+      <c r="F23" s="5">
+        <v>14.549028</v>
+      </c>
+      <c r="G23" s="5">
+        <v>1.2516811000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" s="5">
+        <v>11125.829</v>
+      </c>
+      <c r="C24" s="5">
+        <v>34</v>
+      </c>
+      <c r="D24" s="5">
+        <v>11125.857</v>
+      </c>
+      <c r="E24" s="5">
+        <v>42283.55</v>
+      </c>
+      <c r="F24" s="5">
+        <v>14.671536</v>
+      </c>
+      <c r="G24" s="5">
+        <v>1.2064341999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25" s="5">
+        <v>11454.882</v>
+      </c>
+      <c r="C25" s="5">
+        <v>35</v>
+      </c>
+      <c r="D25" s="5">
+        <v>11454.893</v>
+      </c>
+      <c r="E25" s="5">
+        <v>49571.77</v>
+      </c>
+      <c r="F25" s="5">
+        <v>14.789472</v>
+      </c>
+      <c r="G25" s="5">
+        <v>1.4143817000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" s="5">
+        <v>11783.933999999999</v>
+      </c>
+      <c r="C26" s="5">
+        <v>36</v>
+      </c>
+      <c r="D26" s="5">
+        <v>11783.945</v>
+      </c>
+      <c r="E26" s="5">
+        <v>46799.37</v>
+      </c>
+      <c r="F26" s="5">
+        <v>14.907384</v>
+      </c>
+      <c r="G26" s="5">
+        <v>1.3352796</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" s="5">
+        <v>12112.986999999999</v>
+      </c>
+      <c r="C27" s="5">
+        <v>37</v>
+      </c>
+      <c r="D27" s="5">
+        <v>12113.002</v>
+      </c>
+      <c r="E27" s="5">
+        <v>45605.74</v>
+      </c>
+      <c r="F27" s="5">
+        <v>15.029779</v>
+      </c>
+      <c r="G27" s="5">
+        <v>1.3012229</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B28" s="5">
+        <v>12442.039000000001</v>
+      </c>
+      <c r="C28" s="5">
+        <v>38</v>
+      </c>
+      <c r="D28" s="5">
+        <v>12442.064</v>
+      </c>
+      <c r="E28" s="5">
+        <v>39608.410000000003</v>
+      </c>
+      <c r="F28" s="5">
+        <v>15.152137</v>
+      </c>
+      <c r="G28" s="5">
+        <v>1.1301071</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B29" s="5">
+        <v>12771.092000000001</v>
+      </c>
+      <c r="C29" s="5">
+        <v>39</v>
+      </c>
+      <c r="D29" s="5">
+        <v>12771.091</v>
+      </c>
+      <c r="E29" s="5">
+        <v>42492.08</v>
+      </c>
+      <c r="F29" s="5">
+        <v>15.242755000000001</v>
+      </c>
+      <c r="G29" s="5">
+        <v>1.2123839999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B30" s="5">
+        <v>13100.144</v>
+      </c>
+      <c r="C30" s="5">
+        <v>40</v>
+      </c>
+      <c r="D30" s="5">
+        <v>13100.152</v>
+      </c>
+      <c r="E30" s="5">
+        <v>40449.730000000003</v>
+      </c>
+      <c r="F30" s="5">
+        <v>15.360554</v>
+      </c>
+      <c r="G30" s="5">
+        <v>1.1541116</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B31" s="5">
+        <v>13429.197</v>
+      </c>
+      <c r="C31" s="5">
+        <v>41</v>
+      </c>
+      <c r="D31" s="5">
+        <v>13429.221</v>
+      </c>
+      <c r="E31" s="5">
+        <v>41194.53</v>
+      </c>
+      <c r="F31" s="5">
+        <v>15.451152</v>
+      </c>
+      <c r="G31" s="5">
+        <v>1.1753623</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B32" s="5">
+        <v>13758.249</v>
+      </c>
+      <c r="C32" s="5">
+        <v>42</v>
+      </c>
+      <c r="D32" s="5">
+        <v>13758.252</v>
+      </c>
+      <c r="E32" s="5">
+        <v>44226.720000000001</v>
+      </c>
+      <c r="F32" s="5">
+        <v>15.541733000000001</v>
+      </c>
+      <c r="G32" s="5">
+        <v>1.2618767</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A33" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B33" s="5">
+        <v>14087.302</v>
+      </c>
+      <c r="C33" s="5">
+        <v>43</v>
+      </c>
+      <c r="D33" s="5">
+        <v>14087.31</v>
+      </c>
+      <c r="E33" s="5">
+        <v>42654.36</v>
+      </c>
+      <c r="F33" s="5">
+        <v>15.63227</v>
+      </c>
+      <c r="G33" s="5">
+        <v>1.2170141000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A34" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B34" s="5">
+        <v>14416.353999999999</v>
+      </c>
+      <c r="C34" s="5">
+        <v>44</v>
+      </c>
+      <c r="D34" s="5">
+        <v>14416.371999999999</v>
+      </c>
+      <c r="E34" s="5">
+        <v>45347.3</v>
+      </c>
+      <c r="F34" s="5">
+        <v>15.691098</v>
+      </c>
+      <c r="G34" s="5">
+        <v>1.2938491000000001</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A35" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B35" s="5">
+        <v>14745.406999999999</v>
+      </c>
+      <c r="C35" s="5">
+        <v>45</v>
+      </c>
+      <c r="D35" s="5">
+        <v>14745.438</v>
+      </c>
+      <c r="E35" s="5">
+        <v>39091.26</v>
+      </c>
+      <c r="F35" s="5">
+        <v>15.77707</v>
+      </c>
+      <c r="G35" s="5">
+        <v>1.1153518</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A36" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B36" s="5">
+        <v>15074.459000000001</v>
+      </c>
+      <c r="C36" s="5">
+        <v>46</v>
+      </c>
+      <c r="D36" s="5">
+        <v>15074.478999999999</v>
+      </c>
+      <c r="E36" s="5">
+        <v>46242.15</v>
+      </c>
+      <c r="F36" s="5">
+        <v>15.867528999999999</v>
+      </c>
+      <c r="G36" s="5">
+        <v>1.3193809999999999</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A37" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B37" s="5">
+        <v>15403.512000000001</v>
+      </c>
+      <c r="C37" s="5">
+        <v>47</v>
+      </c>
+      <c r="D37" s="5">
+        <v>15403.536</v>
+      </c>
+      <c r="E37" s="5">
+        <v>42224.54</v>
+      </c>
+      <c r="F37" s="5">
+        <v>15.930849</v>
+      </c>
+      <c r="G37" s="5">
+        <v>1.2047505000000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A38" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B38" s="5">
+        <v>15732.564</v>
+      </c>
+      <c r="C38" s="5">
+        <v>48</v>
+      </c>
+      <c r="D38" s="5">
+        <v>15732.587</v>
+      </c>
+      <c r="E38" s="5">
+        <v>45765.48</v>
+      </c>
+      <c r="F38" s="5">
+        <v>16.021315000000001</v>
+      </c>
+      <c r="G38" s="5">
+        <v>1.3057806000000001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A39" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B39" s="5">
+        <v>16061.617</v>
+      </c>
+      <c r="C39" s="5">
+        <v>49</v>
+      </c>
+      <c r="D39" s="5">
+        <v>16061.641</v>
+      </c>
+      <c r="E39" s="5">
+        <v>46698.02</v>
+      </c>
+      <c r="F39" s="5">
+        <v>16.080110999999999</v>
+      </c>
+      <c r="G39" s="5">
+        <v>1.3323878</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A40" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B40" s="5">
+        <v>16390.669000000002</v>
+      </c>
+      <c r="C40" s="5">
+        <v>50</v>
+      </c>
+      <c r="D40" s="5">
+        <v>16390.691999999999</v>
+      </c>
+      <c r="E40" s="5">
+        <v>41276.54</v>
+      </c>
+      <c r="F40" s="5">
+        <v>16.138932</v>
+      </c>
+      <c r="G40" s="5">
+        <v>1.1777021999999999</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A41" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B41" s="5">
+        <v>16719.722000000002</v>
+      </c>
+      <c r="C41" s="5">
+        <v>51</v>
+      </c>
+      <c r="D41" s="5">
+        <v>16719.732</v>
+      </c>
+      <c r="E41" s="5">
+        <v>42050.73</v>
+      </c>
+      <c r="F41" s="5">
+        <v>16.202285</v>
+      </c>
+      <c r="G41" s="5">
+        <v>1.1997914000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A42" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B42" s="5">
+        <v>17048.774000000001</v>
+      </c>
+      <c r="C42" s="5">
+        <v>52</v>
+      </c>
+      <c r="D42" s="5">
+        <v>17048.794999999998</v>
+      </c>
+      <c r="E42" s="5">
+        <v>42524.17</v>
+      </c>
+      <c r="F42" s="5">
+        <v>16.292787000000001</v>
+      </c>
+      <c r="G42" s="5">
+        <v>1.2132996</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A43" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B43" s="5">
+        <v>17377.827000000001</v>
+      </c>
+      <c r="C43" s="5">
+        <v>53</v>
+      </c>
+      <c r="D43" s="5">
+        <v>17377.852999999999</v>
+      </c>
+      <c r="E43" s="5">
+        <v>40384.660000000003</v>
+      </c>
+      <c r="F43" s="5">
+        <v>16.319941</v>
+      </c>
+      <c r="G43" s="5">
+        <v>1.1522551000000001</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A44" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B44" s="5">
+        <v>17706.879000000001</v>
+      </c>
+      <c r="C44" s="5">
+        <v>54</v>
+      </c>
+      <c r="D44" s="5">
+        <v>17706.902999999998</v>
+      </c>
+      <c r="E44" s="5">
+        <v>44038.34</v>
+      </c>
+      <c r="F44" s="5">
+        <v>16.383289999999999</v>
+      </c>
+      <c r="G44" s="5">
+        <v>1.2565018999999999</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A45" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B45" s="5">
+        <v>18035.932000000001</v>
+      </c>
+      <c r="C45" s="5">
+        <v>55</v>
+      </c>
+      <c r="D45" s="5">
+        <v>18035.942999999999</v>
+      </c>
+      <c r="E45" s="5">
+        <v>39107.22</v>
+      </c>
+      <c r="F45" s="5">
+        <v>16.437601999999998</v>
+      </c>
+      <c r="G45" s="5">
+        <v>1.1158071000000001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A46" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B46" s="5">
+        <v>18364.984</v>
+      </c>
+      <c r="C46" s="5">
+        <v>56</v>
+      </c>
+      <c r="D46" s="5">
+        <v>18365.004000000001</v>
+      </c>
+      <c r="E46" s="5">
+        <v>18154.349999999999</v>
+      </c>
+      <c r="F46" s="5">
+        <v>16.469287999999999</v>
+      </c>
+      <c r="G46" s="5">
+        <v>0.51797990000000005</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A47" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B47" s="5">
+        <v>18694.037</v>
+      </c>
+      <c r="C47" s="5">
+        <v>57</v>
+      </c>
+      <c r="D47" s="5">
+        <v>18694.059000000001</v>
+      </c>
+      <c r="E47" s="5">
+        <v>35227.589999999997</v>
+      </c>
+      <c r="F47" s="5">
+        <v>16.559826999999999</v>
+      </c>
+      <c r="G47" s="5">
+        <v>1.0051136000000001</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A48" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B48" s="5">
+        <v>19023.089</v>
+      </c>
+      <c r="C48" s="5">
+        <v>58</v>
+      </c>
+      <c r="D48" s="5">
+        <v>19023.116000000002</v>
+      </c>
+      <c r="E48" s="5">
+        <v>27716.54</v>
+      </c>
+      <c r="F48" s="5">
+        <v>16.591521</v>
+      </c>
+      <c r="G48" s="5">
+        <v>0.79080830000000002</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A49" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B49" s="5">
+        <v>19352.142</v>
+      </c>
+      <c r="C49" s="5">
+        <v>59</v>
+      </c>
+      <c r="D49" s="5">
+        <v>19352.169000000002</v>
+      </c>
+      <c r="E49" s="5">
+        <v>24359.79</v>
+      </c>
+      <c r="F49" s="5">
+        <v>16.650390000000002</v>
+      </c>
+      <c r="G49" s="5">
+        <v>0.69503349999999997</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A50" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B50" s="5">
+        <v>19681.194</v>
+      </c>
+      <c r="C50" s="5">
+        <v>60</v>
+      </c>
+      <c r="D50" s="5">
+        <v>19681.218000000001</v>
+      </c>
+      <c r="E50" s="5">
+        <v>14653.88</v>
+      </c>
+      <c r="F50" s="5">
+        <v>16.70926</v>
+      </c>
+      <c r="G50" s="5">
+        <v>0.41810449999999999</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A51" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B51" s="5">
+        <v>20010.246999999999</v>
+      </c>
+      <c r="C51" s="5">
+        <v>61</v>
+      </c>
+      <c r="D51" s="5">
+        <v>20010.271000000001</v>
+      </c>
+      <c r="E51" s="5">
+        <v>6033.57</v>
+      </c>
+      <c r="F51" s="5">
+        <v>16.682086000000002</v>
+      </c>
+      <c r="G51" s="5">
+        <v>0.17214979999999999</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A52" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B52" s="5">
+        <v>20339.298999999999</v>
+      </c>
+      <c r="C52" s="5">
+        <v>62</v>
+      </c>
+      <c r="D52" s="5">
+        <v>20339.311000000002</v>
+      </c>
+      <c r="E52" s="5">
+        <v>18374.14</v>
+      </c>
+      <c r="F52" s="5">
+        <v>16.772684000000002</v>
+      </c>
+      <c r="G52" s="5">
+        <v>0.52425089999999996</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A53" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B53" s="5">
+        <v>20668.351999999999</v>
+      </c>
+      <c r="C53" s="5">
+        <v>63</v>
+      </c>
+      <c r="D53" s="5">
+        <v>20668.38</v>
+      </c>
+      <c r="E53" s="5">
+        <v>18447.060000000001</v>
+      </c>
+      <c r="F53" s="5">
+        <v>16.827065999999999</v>
+      </c>
+      <c r="G53" s="5">
+        <v>0.52633149999999995</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A54" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B54" s="5">
+        <v>20997.403999999999</v>
+      </c>
+      <c r="C54" s="5">
+        <v>64</v>
+      </c>
+      <c r="D54" s="5">
+        <v>20997.417000000001</v>
+      </c>
+      <c r="E54" s="5">
+        <v>16611.09</v>
+      </c>
+      <c r="F54" s="5">
+        <v>16.863329</v>
+      </c>
+      <c r="G54" s="5">
+        <v>0.47394760000000002</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A55" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B55" s="5">
+        <v>21326.456999999999</v>
+      </c>
+      <c r="C55" s="5">
+        <v>65</v>
+      </c>
+      <c r="D55" s="5">
+        <v>21326.477999999999</v>
+      </c>
+      <c r="E55" s="5">
+        <v>16524.68</v>
+      </c>
+      <c r="F55" s="5">
+        <v>16.917757999999999</v>
+      </c>
+      <c r="G55" s="5">
+        <v>0.47148210000000002</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A56" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B56" s="5">
+        <v>21655.508999999998</v>
+      </c>
+      <c r="C56" s="5">
+        <v>66</v>
+      </c>
+      <c r="D56" s="5">
+        <v>21655.525000000001</v>
+      </c>
+      <c r="E56" s="5">
+        <v>5806.63</v>
+      </c>
+      <c r="F56" s="5">
+        <v>16.890540999999999</v>
+      </c>
+      <c r="G56" s="5">
+        <v>0.16567480000000001</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" s="3" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B57" s="6">
+        <v>23300.772000000001</v>
+      </c>
+      <c r="C57" s="6">
+        <v>71</v>
+      </c>
+      <c r="D57" s="6">
+        <v>23300.761999999999</v>
+      </c>
+      <c r="E57" s="6">
+        <v>11896.52</v>
+      </c>
+      <c r="F57" s="6">
+        <v>17.099250000000001</v>
+      </c>
+      <c r="G57" s="6">
+        <v>0.3394315</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2DA3A05-A028-4146-99E0-71BDBFA6D7F2}">
+  <dimension ref="A1:G30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="5">
+        <v>1334.2249999999999</v>
+      </c>
+      <c r="C2" s="5">
+        <v>4</v>
+      </c>
+      <c r="D2" s="5">
+        <v>1334.221</v>
+      </c>
+      <c r="E2" s="5">
+        <v>316411.02</v>
+      </c>
+      <c r="F2" s="5">
+        <v>0.89764949999999999</v>
+      </c>
+      <c r="G2" s="5">
+        <v>9.0278387999999996</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="5">
+        <v>1663.277</v>
+      </c>
+      <c r="C3" s="5">
+        <v>5</v>
+      </c>
+      <c r="D3" s="5">
+        <v>1663.2750000000001</v>
+      </c>
+      <c r="E3" s="5">
+        <v>188402.51</v>
+      </c>
+      <c r="F3" s="5">
+        <v>1.1415884999999999</v>
+      </c>
+      <c r="G3" s="5">
+        <v>5.3755001599999996</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="5">
+        <v>1992.33</v>
+      </c>
+      <c r="C4" s="5">
+        <v>6</v>
+      </c>
+      <c r="D4" s="5">
+        <v>1992.329</v>
+      </c>
+      <c r="E4" s="5">
+        <v>142149.94</v>
+      </c>
+      <c r="F4" s="5">
+        <v>1.8915002999999999</v>
+      </c>
+      <c r="G4" s="5">
+        <v>4.0558218999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="5">
+        <v>2321.3820000000001</v>
+      </c>
+      <c r="C5" s="5">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5">
+        <v>2321.38</v>
+      </c>
+      <c r="E5" s="5">
+        <v>97016.71</v>
+      </c>
+      <c r="F5" s="5">
+        <v>3.4500158999999999</v>
+      </c>
+      <c r="G5" s="5">
+        <v>2.76808064</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="5">
+        <v>2650.4349999999999</v>
+      </c>
+      <c r="C6" s="5">
+        <v>8</v>
+      </c>
+      <c r="D6" s="5">
+        <v>2650.433</v>
+      </c>
+      <c r="E6" s="5">
+        <v>125682.29</v>
+      </c>
+      <c r="F6" s="5">
+        <v>4.8010088</v>
+      </c>
+      <c r="G6" s="5">
+        <v>3.5859669300000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="5">
+        <v>2979.4870000000001</v>
+      </c>
+      <c r="C7" s="5">
+        <v>9</v>
+      </c>
+      <c r="D7" s="5">
+        <v>2979.4850000000001</v>
+      </c>
+      <c r="E7" s="5">
+        <v>82796.47</v>
+      </c>
+      <c r="F7" s="5">
+        <v>5.9398688000000002</v>
+      </c>
+      <c r="G7" s="5">
+        <v>2.3623487700000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="5">
+        <v>3308.54</v>
+      </c>
+      <c r="C8" s="5">
+        <v>10</v>
+      </c>
+      <c r="D8" s="5">
+        <v>3308.54</v>
+      </c>
+      <c r="E8" s="5">
+        <v>41816.620000000003</v>
+      </c>
+      <c r="F8" s="5">
+        <v>6.8711072</v>
+      </c>
+      <c r="G8" s="5">
+        <v>1.1931117499999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="5">
+        <v>3637.5920000000001</v>
+      </c>
+      <c r="C9" s="5">
+        <v>11</v>
+      </c>
+      <c r="D9" s="5">
+        <v>3637.596</v>
+      </c>
+      <c r="E9" s="5">
+        <v>35762.19</v>
+      </c>
+      <c r="F9" s="5">
+        <v>7.6490736999999998</v>
+      </c>
+      <c r="G9" s="5">
+        <v>1.0203667599999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5">
+        <v>4624.75</v>
+      </c>
+      <c r="C10" s="5">
+        <v>14</v>
+      </c>
+      <c r="D10" s="5">
+        <v>4624.7659999999996</v>
+      </c>
+      <c r="E10" s="5">
+        <v>28286.81</v>
+      </c>
+      <c r="F10" s="5">
+        <v>9.4788820999999999</v>
+      </c>
+      <c r="G10" s="5">
+        <v>0.80707921999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="5">
+        <v>4953.8019999999997</v>
+      </c>
+      <c r="C11" s="5">
+        <v>15</v>
+      </c>
+      <c r="D11" s="5">
+        <v>4953.8119999999999</v>
+      </c>
+      <c r="E11" s="5">
+        <v>39444.54</v>
+      </c>
+      <c r="F11" s="5">
+        <v>9.9594076999999999</v>
+      </c>
+      <c r="G11" s="5">
+        <v>1.12543156</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="5">
+        <v>5282.8549999999996</v>
+      </c>
+      <c r="C12" s="5">
+        <v>16</v>
+      </c>
+      <c r="D12" s="5">
+        <v>5282.8559999999998</v>
+      </c>
+      <c r="E12" s="5">
+        <v>79399.44</v>
+      </c>
+      <c r="F12" s="5">
+        <v>10.4401247</v>
+      </c>
+      <c r="G12" s="5">
+        <v>2.2654247199999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="5">
+        <v>5611.9070000000002</v>
+      </c>
+      <c r="C13" s="5">
+        <v>17</v>
+      </c>
+      <c r="D13" s="5">
+        <v>5611.9179999999997</v>
+      </c>
+      <c r="E13" s="5">
+        <v>85549.16</v>
+      </c>
+      <c r="F13" s="5">
+        <v>10.857465299999999</v>
+      </c>
+      <c r="G13" s="5">
+        <v>2.4408885200000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="5">
+        <v>9889.59</v>
+      </c>
+      <c r="C14" s="5">
+        <v>30</v>
+      </c>
+      <c r="D14" s="5">
+        <v>9889.5840000000007</v>
+      </c>
+      <c r="E14" s="5">
+        <v>20427.64</v>
+      </c>
+      <c r="F14" s="5">
+        <v>14.072015</v>
+      </c>
+      <c r="G14" s="5">
+        <v>0.58284139999999995</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" s="5">
+        <v>10218.642</v>
+      </c>
+      <c r="C15" s="5">
+        <v>31</v>
+      </c>
+      <c r="D15" s="5">
+        <v>10218.662</v>
+      </c>
+      <c r="E15" s="5">
+        <v>17533.73</v>
+      </c>
+      <c r="F15" s="5">
+        <v>14.2492003</v>
+      </c>
+      <c r="G15" s="5">
+        <v>0.50027235999999997</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="5">
+        <v>11205.8</v>
+      </c>
+      <c r="C16" s="5">
+        <v>34</v>
+      </c>
+      <c r="D16" s="5">
+        <v>11205.807000000001</v>
+      </c>
+      <c r="E16" s="5">
+        <v>12936.37</v>
+      </c>
+      <c r="F16" s="5">
+        <v>14.671536400000001</v>
+      </c>
+      <c r="G16" s="5">
+        <v>0.36910049</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="5">
+        <v>11863.905000000001</v>
+      </c>
+      <c r="C17" s="5">
+        <v>36</v>
+      </c>
+      <c r="D17" s="5">
+        <v>11863.925999999999</v>
+      </c>
+      <c r="E17" s="5">
+        <v>14120.57</v>
+      </c>
+      <c r="F17" s="5">
+        <v>14.907383899999999</v>
+      </c>
+      <c r="G17" s="5">
+        <v>0.40288807999999998</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="5">
+        <v>12522.01</v>
+      </c>
+      <c r="C18" s="5">
+        <v>38</v>
+      </c>
+      <c r="D18" s="5">
+        <v>12522.012000000001</v>
+      </c>
+      <c r="E18" s="5">
+        <v>15992.18</v>
+      </c>
+      <c r="F18" s="5">
+        <v>15.1204106</v>
+      </c>
+      <c r="G18" s="5">
+        <v>0.45628886000000002</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" s="5">
+        <v>13509.166999999999</v>
+      </c>
+      <c r="C19" s="5">
+        <v>41</v>
+      </c>
+      <c r="D19" s="5">
+        <v>13509.161</v>
+      </c>
+      <c r="E19" s="5">
+        <v>12568.7</v>
+      </c>
+      <c r="F19" s="5">
+        <v>15.387741999999999</v>
+      </c>
+      <c r="G19" s="5">
+        <v>0.35861013000000003</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="5">
+        <v>13838.22</v>
+      </c>
+      <c r="C20" s="5">
+        <v>42</v>
+      </c>
+      <c r="D20" s="5">
+        <v>13838.201999999999</v>
+      </c>
+      <c r="E20" s="5">
+        <v>11491.94</v>
+      </c>
+      <c r="F20" s="5">
+        <v>15.478327200000001</v>
+      </c>
+      <c r="G20" s="5">
+        <v>0.32788802</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21" s="5">
+        <v>14167.272000000001</v>
+      </c>
+      <c r="C21" s="5">
+        <v>43</v>
+      </c>
+      <c r="D21" s="5">
+        <v>14167.261</v>
+      </c>
+      <c r="E21" s="5">
+        <v>11573.17</v>
+      </c>
+      <c r="F21" s="5">
+        <v>15.6005691</v>
+      </c>
+      <c r="G21" s="5">
+        <v>0.33020567000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" s="5">
+        <v>14496.325000000001</v>
+      </c>
+      <c r="C22" s="5">
+        <v>44</v>
+      </c>
+      <c r="D22" s="5">
+        <v>14496.343999999999</v>
+      </c>
+      <c r="E22" s="5">
+        <v>10378.23</v>
+      </c>
+      <c r="F22" s="5">
+        <v>15.6594251</v>
+      </c>
+      <c r="G22" s="5">
+        <v>0.29611164000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="5">
+        <v>14825.377</v>
+      </c>
+      <c r="C23" s="5">
+        <v>45</v>
+      </c>
+      <c r="D23" s="5">
+        <v>14825.371999999999</v>
+      </c>
+      <c r="E23" s="5">
+        <v>10751.65</v>
+      </c>
+      <c r="F23" s="5">
+        <v>15.749924200000001</v>
+      </c>
+      <c r="G23" s="5">
+        <v>0.30676606000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" s="5">
+        <v>15154.43</v>
+      </c>
+      <c r="C24" s="5">
+        <v>46</v>
+      </c>
+      <c r="D24" s="5">
+        <v>15154.422</v>
+      </c>
+      <c r="E24" s="5">
+        <v>8975.32</v>
+      </c>
+      <c r="F24" s="5">
+        <v>15.813253899999999</v>
+      </c>
+      <c r="G24" s="5">
+        <v>0.25608382000000002</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25" s="5">
+        <v>15483.482</v>
+      </c>
+      <c r="C25" s="5">
+        <v>47</v>
+      </c>
+      <c r="D25" s="5">
+        <v>15483.473</v>
+      </c>
+      <c r="E25" s="5">
+        <v>8714.7999999999993</v>
+      </c>
+      <c r="F25" s="5">
+        <v>15.8991948</v>
+      </c>
+      <c r="G25" s="5">
+        <v>0.24865066</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" s="5">
+        <v>16470.64</v>
+      </c>
+      <c r="C26" s="5">
+        <v>50</v>
+      </c>
+      <c r="D26" s="5">
+        <v>16470.624</v>
+      </c>
+      <c r="E26" s="5">
+        <v>7660.03</v>
+      </c>
+      <c r="F26" s="5">
+        <v>16.111785399999999</v>
+      </c>
+      <c r="G26" s="5">
+        <v>0.21855596999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" s="5">
+        <v>16799.691999999999</v>
+      </c>
+      <c r="C27" s="5">
+        <v>51</v>
+      </c>
+      <c r="D27" s="5">
+        <v>16799.7</v>
+      </c>
+      <c r="E27" s="5">
+        <v>5237.6400000000003</v>
+      </c>
+      <c r="F27" s="5">
+        <v>16.1706121</v>
+      </c>
+      <c r="G27" s="5">
+        <v>0.14944034</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B28" s="5">
+        <v>17457.796999999999</v>
+      </c>
+      <c r="C28" s="5">
+        <v>53</v>
+      </c>
+      <c r="D28" s="5">
+        <v>17457.803</v>
+      </c>
+      <c r="E28" s="5">
+        <v>8023.21</v>
+      </c>
+      <c r="F28" s="5">
+        <v>16.292787000000001</v>
+      </c>
+      <c r="G28" s="5">
+        <v>0.22891822000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B29" s="5">
+        <v>18115.902999999998</v>
+      </c>
+      <c r="C29" s="5">
+        <v>55</v>
+      </c>
+      <c r="D29" s="5">
+        <v>18115.911</v>
+      </c>
+      <c r="E29" s="5">
+        <v>5947.27</v>
+      </c>
+      <c r="F29" s="5">
+        <v>16.383289900000001</v>
+      </c>
+      <c r="G29" s="5">
+        <v>0.16968749999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B30" s="5">
+        <v>18444.955000000002</v>
+      </c>
+      <c r="C30" s="5">
+        <v>56</v>
+      </c>
+      <c r="D30" s="5">
+        <v>18444.937000000002</v>
+      </c>
+      <c r="E30" s="5">
+        <v>3174.69</v>
+      </c>
+      <c r="F30" s="5">
+        <v>16.437601600000001</v>
+      </c>
+      <c r="G30" s="5">
+        <v>9.0580250000000001E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09756682-BD63-1F40-A48C-591EE184884F}">
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B2">
+        <v>309.79160000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="5">
+        <v>7877.9989999999998</v>
+      </c>
+      <c r="D3" s="5">
+        <v>23</v>
+      </c>
+      <c r="E3" s="5">
+        <v>7877.9989999999998</v>
+      </c>
+      <c r="F3" s="5">
+        <v>33101.31</v>
+      </c>
+      <c r="G3" s="5">
+        <v>9.9594079999999998</v>
+      </c>
+      <c r="H3" s="5">
+        <v>0.94444649999999997</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="5">
+        <v>8207.0519999999997</v>
+      </c>
+      <c r="D4" s="5">
+        <v>24</v>
+      </c>
+      <c r="E4" s="5">
+        <v>8207.0409999999993</v>
+      </c>
+      <c r="F4" s="5">
+        <v>43693.04</v>
+      </c>
+      <c r="G4" s="5">
+        <v>10.258682</v>
+      </c>
+      <c r="H4" s="5">
+        <v>1.2466497999999999</v>
+      </c>
+      <c r="I4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="5">
+        <v>10839.472</v>
+      </c>
+      <c r="D5" s="5">
+        <v>32</v>
+      </c>
+      <c r="E5" s="5">
+        <v>10839.385</v>
+      </c>
+      <c r="F5" s="5">
+        <v>36479.660000000003</v>
+      </c>
+      <c r="G5" s="5">
+        <v>11.883118</v>
+      </c>
+      <c r="H5" s="5">
+        <v>1.0408375999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="5">
+        <v>11826.629000000001</v>
+      </c>
+      <c r="D6" s="5">
+        <v>35</v>
+      </c>
+      <c r="E6" s="5">
+        <v>11826.562</v>
+      </c>
+      <c r="F6" s="5">
+        <v>58194.6</v>
+      </c>
+      <c r="G6" s="5">
+        <v>12.328101999999999</v>
+      </c>
+      <c r="H6" s="5">
+        <v>1.6604082</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="5">
+        <v>16104.312</v>
+      </c>
+      <c r="D7" s="5">
+        <v>48</v>
+      </c>
+      <c r="E7" s="5">
+        <v>16104.397999999999</v>
+      </c>
+      <c r="F7" s="5">
+        <v>9301.17</v>
+      </c>
+      <c r="G7" s="5">
+        <v>14.970840000000001</v>
+      </c>
+      <c r="H7" s="5">
+        <v>0.26538099999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B10">
+        <v>252.87039999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="4"/>
+      <c r="B11" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="5">
+        <v>3543.395</v>
+      </c>
+      <c r="D11" s="5">
+        <v>10</v>
+      </c>
+      <c r="E11" s="5">
+        <v>3543.4259999999999</v>
+      </c>
+      <c r="F11" s="5">
+        <v>36992.699999999997</v>
+      </c>
+      <c r="G11" s="5">
+        <v>3.6623429999999999</v>
+      </c>
+      <c r="H11" s="5">
+        <v>1.0554756999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="4"/>
+      <c r="B12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="5">
+        <v>3872.4479999999999</v>
+      </c>
+      <c r="D12" s="5">
+        <v>11</v>
+      </c>
+      <c r="E12" s="5">
+        <v>3872.4769999999999</v>
+      </c>
+      <c r="F12" s="5">
+        <v>137053.81</v>
+      </c>
+      <c r="G12" s="5">
+        <v>4.9184970000000003</v>
+      </c>
+      <c r="H12" s="5">
+        <v>3.9104190999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="4"/>
+      <c r="B13" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="5">
+        <v>4859.6049999999996</v>
+      </c>
+      <c r="D13" s="5">
+        <v>14</v>
+      </c>
+      <c r="E13" s="5">
+        <v>4859.6369999999997</v>
+      </c>
+      <c r="F13" s="5">
+        <v>39249.33</v>
+      </c>
+      <c r="G13" s="5">
+        <v>6.1206649999999998</v>
+      </c>
+      <c r="H13" s="5">
+        <v>1.1198618</v>
+      </c>
+      <c r="I13" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="4"/>
+      <c r="B14" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="5">
+        <v>6833.92</v>
+      </c>
+      <c r="D14" s="5">
+        <v>20</v>
+      </c>
+      <c r="E14" s="5">
+        <v>6833.9189999999999</v>
+      </c>
+      <c r="F14" s="5">
+        <v>15432.52</v>
+      </c>
+      <c r="G14" s="5">
+        <v>9.2976039999999998</v>
+      </c>
+      <c r="H14" s="5">
+        <v>0.44032060000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="4"/>
+      <c r="B15" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="5">
+        <v>7162.973</v>
+      </c>
+      <c r="D15" s="5">
+        <v>21</v>
+      </c>
+      <c r="E15" s="5">
+        <v>7162.9740000000002</v>
+      </c>
+      <c r="F15" s="5">
+        <v>9354.43</v>
+      </c>
+      <c r="G15" s="5">
+        <v>9.6329750000000001</v>
+      </c>
+      <c r="H15" s="5">
+        <v>0.26690059999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>